<commit_message>
chore: add v2e working registry analysis assets
</commit_message>
<xml_diff>
--- a/PPP_empirical_reinforcement_bundle_20260416_unified_v3/00_unified_baseline_reference/tables/unified_baseline_reference.xlsx
+++ b/PPP_empirical_reinforcement_bundle_20260416_unified_v3/00_unified_baseline_reference/tables/unified_baseline_reference.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="manuscript_baseline" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="audit_rerun" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spec_anchor" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="manuscript_baseline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="audit_rerun" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="spec_anchor" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -803,13 +803,13 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>0.522638660137449</v>
+        <v>0.5226386601375361</v>
       </c>
       <c r="L2" t="n">
-        <v>0.4515038167814193</v>
+        <v>0.4515038174707404</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2561807054468387</v>
+        <v>0.2561807061571288</v>
       </c>
       <c r="N2" t="n">
         <v>262</v>
@@ -836,13 +836,13 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>-0.002658275457950499</v>
+        <v>-0.002658275457863346</v>
       </c>
       <c r="U2" t="n">
-        <v>0.03010613231362019</v>
+        <v>0.03010613300294124</v>
       </c>
       <c r="V2" t="n">
-        <v>0.04362134003009044</v>
+        <v>0.04362134074038054</v>
       </c>
       <c r="W2" t="b">
         <v>0</v>
@@ -892,13 +892,13 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>0.3599903094733262</v>
+        <v>0.3599903094734115</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1008444514920222</v>
+        <v>0.1008444522409024</v>
       </c>
       <c r="M3" t="n">
-        <v>0.001226450152890302</v>
+        <v>0.001226450239716637</v>
       </c>
       <c r="N3" t="n">
         <v>262</v>
@@ -925,13 +925,13 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>0.004362604720685337</v>
+        <v>0.004362604720770713</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0006808384939146206</v>
+        <v>0.0006808392427948146</v>
       </c>
       <c r="V3" t="n">
-        <v>0.0008419033006828024</v>
+        <v>0.0008419033875091372</v>
       </c>
       <c r="W3" t="b">
         <v>0</v>
@@ -981,13 +981,13 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>-0.4065371976358462</v>
+        <v>-0.4065371976359414</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1022965714861835</v>
+        <v>0.1022965722632587</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0004099922668987794</v>
+        <v>0.0004099923008667163</v>
       </c>
       <c r="N4" t="n">
         <v>262</v>
@@ -1014,13 +1014,13 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>-0.004259711543136924</v>
+        <v>-0.004259711543232125</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0003875668296817875</v>
+        <v>0.0003875676067569694</v>
       </c>
       <c r="V4" t="n">
-        <v>0.0003309938560957809</v>
+        <v>0.0003309938900637177</v>
       </c>
       <c r="W4" t="b">
         <v>0</v>

</xml_diff>